<commit_message>
Ajuste bot legalizador simcard
</commit_message>
<xml_diff>
--- a/src/legalizador_kit_contado/legalizador_kit_contado.xlsx
+++ b/src/legalizador_kit_contado/legalizador_kit_contado.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>La activación no puede continuar por las siguientes razones:; IMEI - Identificación Internacional del Equipo Móvil. = p</t>
+          <t>12877INV-021. El IMEI: "353844853851230", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>La activación no puede continuar por las siguientes razones:; ICC_ID - Identificación Tarjeta de Circuito Integrada. = v</t>
+          <t>12877INV-021. El IMEI: "356263631713041", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -585,12 +585,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>* Su Solicitud fue enviada satisfactoriamente para el producto 270 y el MSISDN asignado es 3142470396.</t>
+          <t>12877INV-021. El IMEI: "356305714142372", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Procesado</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>* Su Solicitud fue enviada satisfactoriamente para el producto 270 y el MSISDN asignado es 3142472891.</t>
+          <t>12877INV-021. El IMEI: "861781078739581", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Procesado</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -663,12 +663,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>* Su Solicitud fue enviada satisfactoriamente para el producto 270 y el MSISDN asignado es 3142476736.</t>
+          <t>12877INV-021. El IMEI: "861819072585269", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Procesado</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>* Su Solicitud fue enviada satisfactoriamente para el producto 270 y el MSISDN asignado es 3142479228.</t>
+          <t>12877INV-021. El IMEI: "863391072693244", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Procesado</t>
+          <t>error</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cambio para xpath de menú principal en legalizador
</commit_message>
<xml_diff>
--- a/src/legalizador_kit_contado/legalizador_kit_contado.xlsx
+++ b/src/legalizador_kit_contado/legalizador_kit_contado.xlsx
@@ -745,12 +745,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>* Su Solicitud fue enviada satisfactoriamente para el producto 270 y el MSISDN asignado es 3142481748.</t>
+          <t>Todos los campos obligatorios deben ser diligenciados</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Procesado</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>* Su Solicitud fue enviada satisfactoriamente para el producto 270 y el MSISDN asignado es 3142483033.</t>
+          <t>12877INV-021. El IMEI: "863015070094754", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -864,12 +864,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>* Su Solicitud fue enviada satisfactoriamente para el producto 270 y el MSISDN asignado es 3142485574.</t>
+          <t>12877INV-021. El IMEI: "865698070210849", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Procesado</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -905,12 +905,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>* Su Solicitud fue enviada satisfactoriamente para el producto 270 y el MSISDN asignado es 3142489353.</t>
+          <t>12877INV-021. El IMEI: "865785070131537", no pertenece al distribuidor</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Procesado</t>
+          <t>error</t>
         </is>
       </c>
     </row>

</xml_diff>